<commit_message>
feat: serve document previews, generate informal equipment docs, and sync static assets
</commit_message>
<xml_diff>
--- a/บัญชีรายการและสิ่งอุปกรณ์.xlsx
+++ b/บัญชีรายการและสิ่งอุปกรณ์.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\WEPAPP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2EBAE5E1-A78C-4935-B86D-E44FFF32561A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD2F63A2-E4A3-4DAA-89E8-C09C2DFC411E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="46296" windowHeight="25656" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,6 +18,7 @@
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -405,7 +406,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="32">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -688,19 +689,6 @@
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
       <right style="medium">
         <color indexed="64"/>
       </right>
@@ -776,23 +764,88 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color auto="1"/>
       </left>
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
+      <top style="medium">
+        <color indexed="64"/>
       </top>
-      <bottom/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -804,10 +857,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -826,17 +875,17 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -877,8 +926,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -894,55 +942,70 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1252,120 +1315,120 @@
   <dimension ref="A1:M115"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="21"/>
   <cols>
-    <col min="1" max="1" width="6" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.33203125" style="7" customWidth="1"/>
+    <col min="1" max="1" width="6" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.33203125" style="5" customWidth="1"/>
     <col min="3" max="4" width="9" style="2"/>
     <col min="5" max="5" width="4.44140625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="11.77734375" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.77734375" style="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="4.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.33203125" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.77734375" style="6" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8" style="6" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.109375" style="6" bestFit="1" customWidth="1"/>
     <col min="14" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="11"/>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="11"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
     </row>
     <row r="3" spans="1:13" ht="12" customHeight="1" thickBot="1"/>
     <row r="4" spans="1:13" ht="21.6" thickBot="1">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="43" t="s">
+      <c r="B4" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="43"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="43"/>
-      <c r="F4" s="44" t="s">
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="44" t="s">
+      <c r="G4" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="44" t="s">
+      <c r="H4" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="I4" s="44" t="s">
-        <v>6</v>
-      </c>
-      <c r="J4" s="44" t="s">
+      <c r="I4" s="39" t="s">
+        <v>6</v>
+      </c>
+      <c r="J4" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="44" t="s">
+      <c r="K4" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="L4" s="44" t="s">
+      <c r="L4" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="M4" s="48" t="s">
+      <c r="M4" s="42" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:13">
-      <c r="A5" s="36">
+      <c r="A5" s="33">
         <v>1</v>
       </c>
-      <c r="B5" s="45" t="s">
+      <c r="B5" s="49" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="45"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="49"/>
-      <c r="G5" s="49"/>
-      <c r="H5" s="49"/>
-      <c r="I5" s="49"/>
-      <c r="J5" s="49"/>
-      <c r="K5" s="49"/>
-      <c r="L5" s="49"/>
-      <c r="M5" s="50"/>
+      <c r="C5" s="49"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="43"/>
+      <c r="I5" s="43"/>
+      <c r="J5" s="43"/>
+      <c r="K5" s="43"/>
+      <c r="L5" s="43"/>
+      <c r="M5" s="44"/>
     </row>
     <row r="6" spans="1:13">
-      <c r="A6" s="36"/>
-      <c r="B6" s="12" t="s">
+      <c r="A6" s="33"/>
+      <c r="B6" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="6"/>
-      <c r="E6" s="13"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="11"/>
       <c r="F6" s="3">
         <v>12</v>
       </c>
@@ -1379,18 +1442,18 @@
       <c r="L6" s="3">
         <v>12</v>
       </c>
-      <c r="M6" s="51"/>
+      <c r="M6" s="45"/>
     </row>
     <row r="7" spans="1:13">
-      <c r="A7" s="36"/>
-      <c r="B7" s="12" t="s">
+      <c r="A7" s="33"/>
+      <c r="B7" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="13"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="11"/>
       <c r="F7" s="3">
         <v>18</v>
       </c>
@@ -1404,18 +1467,18 @@
       <c r="L7" s="3">
         <v>18</v>
       </c>
-      <c r="M7" s="51"/>
+      <c r="M7" s="45"/>
     </row>
     <row r="8" spans="1:13">
-      <c r="A8" s="36"/>
-      <c r="B8" s="12" t="s">
+      <c r="A8" s="33"/>
+      <c r="B8" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="6"/>
-      <c r="E8" s="13"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="11"/>
       <c r="F8" s="3">
         <v>24</v>
       </c>
@@ -1431,18 +1494,18 @@
       <c r="L8" s="3">
         <v>20</v>
       </c>
-      <c r="M8" s="51"/>
+      <c r="M8" s="45"/>
     </row>
     <row r="9" spans="1:13">
-      <c r="A9" s="36"/>
-      <c r="B9" s="12" t="s">
+      <c r="A9" s="33"/>
+      <c r="B9" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="6"/>
-      <c r="E9" s="13"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="11"/>
       <c r="F9" s="3">
         <v>6</v>
       </c>
@@ -1456,18 +1519,18 @@
       <c r="L9" s="3">
         <v>6</v>
       </c>
-      <c r="M9" s="51"/>
+      <c r="M9" s="45"/>
     </row>
     <row r="10" spans="1:13">
-      <c r="A10" s="36">
+      <c r="A10" s="33">
         <v>2</v>
       </c>
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="34"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="35"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="32"/>
       <c r="F10" s="3">
         <v>6</v>
       </c>
@@ -1481,18 +1544,18 @@
       <c r="L10" s="3">
         <v>5</v>
       </c>
-      <c r="M10" s="51"/>
+      <c r="M10" s="45"/>
     </row>
     <row r="11" spans="1:13">
-      <c r="A11" s="36">
+      <c r="A11" s="33">
         <v>3</v>
       </c>
-      <c r="B11" s="29" t="s">
+      <c r="B11" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="34"/>
-      <c r="D11" s="34"/>
-      <c r="E11" s="35"/>
+      <c r="C11" s="30"/>
+      <c r="D11" s="30"/>
+      <c r="E11" s="32"/>
       <c r="F11" s="3">
         <v>6</v>
       </c>
@@ -1506,18 +1569,18 @@
       <c r="L11" s="3">
         <v>6</v>
       </c>
-      <c r="M11" s="51"/>
+      <c r="M11" s="45"/>
     </row>
     <row r="12" spans="1:13">
-      <c r="A12" s="36">
+      <c r="A12" s="33">
         <v>4</v>
       </c>
-      <c r="B12" s="29" t="s">
+      <c r="B12" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="34"/>
-      <c r="D12" s="34"/>
-      <c r="E12" s="35"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="32"/>
       <c r="F12" s="3">
         <v>96</v>
       </c>
@@ -1533,18 +1596,18 @@
       <c r="L12" s="3">
         <v>64</v>
       </c>
-      <c r="M12" s="51"/>
+      <c r="M12" s="45"/>
     </row>
     <row r="13" spans="1:13">
-      <c r="A13" s="36">
+      <c r="A13" s="33">
         <v>5</v>
       </c>
-      <c r="B13" s="26" t="s">
+      <c r="B13" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="13"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="11"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
@@ -1552,18 +1615,18 @@
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
-      <c r="M13" s="51"/>
+      <c r="M13" s="45"/>
     </row>
     <row r="14" spans="1:13">
-      <c r="A14" s="36"/>
-      <c r="B14" s="12" t="s">
+      <c r="A14" s="33"/>
+      <c r="B14" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D14" s="6"/>
-      <c r="E14" s="13"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="11"/>
       <c r="F14" s="3">
         <v>6</v>
       </c>
@@ -1579,18 +1642,18 @@
       <c r="L14" s="3">
         <v>4</v>
       </c>
-      <c r="M14" s="51"/>
+      <c r="M14" s="45"/>
     </row>
     <row r="15" spans="1:13">
-      <c r="A15" s="36"/>
-      <c r="B15" s="12" t="s">
+      <c r="A15" s="33"/>
+      <c r="B15" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D15" s="6"/>
-      <c r="E15" s="13"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="11"/>
       <c r="F15" s="3">
         <v>6</v>
       </c>
@@ -1606,18 +1669,18 @@
       <c r="L15" s="3">
         <v>4</v>
       </c>
-      <c r="M15" s="51"/>
+      <c r="M15" s="45"/>
     </row>
     <row r="16" spans="1:13">
-      <c r="A16" s="36"/>
-      <c r="B16" s="14" t="s">
+      <c r="A16" s="33"/>
+      <c r="B16" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C16" s="15" t="s">
+      <c r="C16" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="15"/>
-      <c r="E16" s="16"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="14"/>
       <c r="F16" s="3">
         <v>6</v>
       </c>
@@ -1633,18 +1696,18 @@
       <c r="L16" s="3">
         <v>4</v>
       </c>
-      <c r="M16" s="51"/>
+      <c r="M16" s="45"/>
     </row>
     <row r="17" spans="1:13">
-      <c r="A17" s="36">
-        <v>6</v>
-      </c>
-      <c r="B17" s="20" t="s">
+      <c r="A17" s="33">
+        <v>6</v>
+      </c>
+      <c r="B17" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="19"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="17"/>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
@@ -1652,18 +1715,18 @@
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
       <c r="L17" s="3"/>
-      <c r="M17" s="51"/>
+      <c r="M17" s="45"/>
     </row>
     <row r="18" spans="1:13">
-      <c r="A18" s="36"/>
-      <c r="B18" s="21" t="s">
+      <c r="A18" s="33"/>
+      <c r="B18" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D18" s="6"/>
-      <c r="E18" s="13"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="11"/>
       <c r="F18" s="3">
         <v>6</v>
       </c>
@@ -1677,18 +1740,18 @@
       <c r="L18" s="3">
         <v>6</v>
       </c>
-      <c r="M18" s="51"/>
+      <c r="M18" s="45"/>
     </row>
     <row r="19" spans="1:13">
-      <c r="A19" s="36"/>
-      <c r="B19" s="21" t="s">
+      <c r="A19" s="33"/>
+      <c r="B19" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D19" s="6"/>
-      <c r="E19" s="13"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="11"/>
       <c r="F19" s="3">
         <v>6</v>
       </c>
@@ -1702,18 +1765,18 @@
       <c r="L19" s="3">
         <v>6</v>
       </c>
-      <c r="M19" s="51"/>
+      <c r="M19" s="45"/>
     </row>
     <row r="20" spans="1:13">
-      <c r="A20" s="36">
+      <c r="A20" s="33">
         <v>7</v>
       </c>
-      <c r="B20" s="29" t="s">
+      <c r="B20" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="34"/>
-      <c r="D20" s="34"/>
-      <c r="E20" s="35"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="32"/>
       <c r="F20" s="3">
         <v>6</v>
       </c>
@@ -1727,18 +1790,18 @@
       <c r="L20" s="3">
         <v>6</v>
       </c>
-      <c r="M20" s="51"/>
+      <c r="M20" s="45"/>
     </row>
     <row r="21" spans="1:13">
-      <c r="A21" s="36">
+      <c r="A21" s="33">
         <v>8</v>
       </c>
-      <c r="B21" s="29" t="s">
+      <c r="B21" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C21" s="34"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="35"/>
+      <c r="C21" s="30"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="32"/>
       <c r="F21" s="3">
         <v>6</v>
       </c>
@@ -1752,18 +1815,18 @@
       <c r="L21" s="3">
         <v>6</v>
       </c>
-      <c r="M21" s="51"/>
+      <c r="M21" s="45"/>
     </row>
     <row r="22" spans="1:13">
-      <c r="A22" s="36">
+      <c r="A22" s="33">
         <v>9</v>
       </c>
-      <c r="B22" s="29" t="s">
+      <c r="B22" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C22" s="34"/>
-      <c r="D22" s="34"/>
-      <c r="E22" s="35"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="32"/>
       <c r="F22" s="3">
         <v>6</v>
       </c>
@@ -1777,18 +1840,18 @@
       <c r="L22" s="3">
         <v>6</v>
       </c>
-      <c r="M22" s="51"/>
+      <c r="M22" s="45"/>
     </row>
     <row r="23" spans="1:13">
-      <c r="A23" s="36">
+      <c r="A23" s="33">
         <v>10</v>
       </c>
-      <c r="B23" s="33" t="s">
+      <c r="B23" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="13"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="11"/>
       <c r="F23" s="3">
         <v>6</v>
       </c>
@@ -1802,18 +1865,18 @@
       <c r="L23" s="3">
         <v>6</v>
       </c>
-      <c r="M23" s="51"/>
+      <c r="M23" s="45"/>
     </row>
     <row r="24" spans="1:13">
-      <c r="A24" s="36"/>
-      <c r="B24" s="12" t="s">
+      <c r="A24" s="33"/>
+      <c r="B24" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D24" s="6"/>
-      <c r="E24" s="13"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="11"/>
       <c r="F24" s="3">
         <v>6</v>
       </c>
@@ -1829,18 +1892,18 @@
       <c r="L24" s="3">
         <v>5</v>
       </c>
-      <c r="M24" s="51"/>
+      <c r="M24" s="45"/>
     </row>
     <row r="25" spans="1:13">
-      <c r="A25" s="36">
+      <c r="A25" s="33">
         <v>11</v>
       </c>
-      <c r="B25" s="29" t="s">
+      <c r="B25" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="34"/>
-      <c r="D25" s="34"/>
-      <c r="E25" s="35"/>
+      <c r="C25" s="30"/>
+      <c r="D25" s="30"/>
+      <c r="E25" s="32"/>
       <c r="F25" s="3">
         <v>6</v>
       </c>
@@ -1856,18 +1919,18 @@
       <c r="L25" s="3">
         <v>4</v>
       </c>
-      <c r="M25" s="51"/>
+      <c r="M25" s="45"/>
     </row>
     <row r="26" spans="1:13">
-      <c r="A26" s="36">
+      <c r="A26" s="33">
         <v>12</v>
       </c>
-      <c r="B26" s="29" t="s">
+      <c r="B26" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="C26" s="30"/>
-      <c r="D26" s="30"/>
-      <c r="E26" s="31"/>
+      <c r="C26" s="28"/>
+      <c r="D26" s="28"/>
+      <c r="E26" s="29"/>
       <c r="F26" s="3">
         <v>60</v>
       </c>
@@ -1883,18 +1946,18 @@
       <c r="L26" s="3">
         <v>40</v>
       </c>
-      <c r="M26" s="51"/>
+      <c r="M26" s="45"/>
     </row>
     <row r="27" spans="1:13">
-      <c r="A27" s="36">
+      <c r="A27" s="33">
         <v>13</v>
       </c>
-      <c r="B27" s="29" t="s">
+      <c r="B27" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="C27" s="30"/>
-      <c r="D27" s="30"/>
-      <c r="E27" s="31"/>
+      <c r="C27" s="28"/>
+      <c r="D27" s="28"/>
+      <c r="E27" s="29"/>
       <c r="F27" s="3">
         <v>12</v>
       </c>
@@ -1910,18 +1973,18 @@
       <c r="L27" s="3">
         <v>4</v>
       </c>
-      <c r="M27" s="51"/>
+      <c r="M27" s="45"/>
     </row>
     <row r="28" spans="1:13">
-      <c r="A28" s="36">
+      <c r="A28" s="33">
         <v>14</v>
       </c>
-      <c r="B28" s="29" t="s">
+      <c r="B28" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="C28" s="30"/>
-      <c r="D28" s="30"/>
-      <c r="E28" s="31"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="28"/>
+      <c r="E28" s="29"/>
       <c r="F28" s="3">
         <v>6</v>
       </c>
@@ -1937,18 +2000,18 @@
       <c r="L28" s="3">
         <v>5</v>
       </c>
-      <c r="M28" s="51"/>
+      <c r="M28" s="45"/>
     </row>
     <row r="29" spans="1:13">
-      <c r="A29" s="36">
+      <c r="A29" s="33">
         <v>15</v>
       </c>
-      <c r="B29" s="29" t="s">
+      <c r="B29" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="C29" s="30"/>
-      <c r="D29" s="30"/>
-      <c r="E29" s="31"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="29"/>
       <c r="F29" s="3">
         <v>6</v>
       </c>
@@ -1964,18 +2027,18 @@
       <c r="L29" s="3">
         <v>4</v>
       </c>
-      <c r="M29" s="51"/>
+      <c r="M29" s="45"/>
     </row>
     <row r="30" spans="1:13">
-      <c r="A30" s="36">
+      <c r="A30" s="33">
         <v>16</v>
       </c>
-      <c r="B30" s="29" t="s">
+      <c r="B30" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="C30" s="30"/>
-      <c r="D30" s="30"/>
-      <c r="E30" s="31"/>
+      <c r="C30" s="28"/>
+      <c r="D30" s="28"/>
+      <c r="E30" s="29"/>
       <c r="F30" s="3">
         <v>12</v>
       </c>
@@ -1989,18 +2052,16 @@
       <c r="L30" s="3">
         <v>12</v>
       </c>
-      <c r="M30" s="51"/>
+      <c r="M30" s="45"/>
     </row>
     <row r="31" spans="1:13">
-      <c r="A31" s="36">
+      <c r="A31" s="33">
         <v>17</v>
       </c>
-      <c r="B31" s="26" t="s">
+      <c r="B31" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="27"/>
+      <c r="E31" s="25"/>
       <c r="F31" s="3">
         <v>6</v>
       </c>
@@ -2016,18 +2077,17 @@
       <c r="L31" s="3">
         <v>4</v>
       </c>
-      <c r="M31" s="51"/>
+      <c r="M31" s="45"/>
     </row>
     <row r="32" spans="1:13">
-      <c r="A32" s="36"/>
-      <c r="B32" s="12" t="s">
+      <c r="A32" s="33"/>
+      <c r="B32" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="C32" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D32" s="5"/>
-      <c r="E32" s="27"/>
+      <c r="E32" s="25"/>
       <c r="F32" s="3">
         <v>6</v>
       </c>
@@ -2043,18 +2103,18 @@
       <c r="L32" s="3">
         <v>4</v>
       </c>
-      <c r="M32" s="51"/>
+      <c r="M32" s="45"/>
     </row>
     <row r="33" spans="1:13">
-      <c r="A33" s="36">
+      <c r="A33" s="33">
         <v>18</v>
       </c>
-      <c r="B33" s="29" t="s">
+      <c r="B33" s="27" t="s">
         <v>37</v>
       </c>
-      <c r="C33" s="30"/>
-      <c r="D33" s="30"/>
-      <c r="E33" s="31"/>
+      <c r="C33" s="28"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="29"/>
       <c r="F33" s="3">
         <v>6</v>
       </c>
@@ -2070,18 +2130,18 @@
       <c r="L33" s="3">
         <v>4</v>
       </c>
-      <c r="M33" s="51"/>
+      <c r="M33" s="45"/>
     </row>
     <row r="34" spans="1:13">
-      <c r="A34" s="36">
+      <c r="A34" s="33">
         <v>19</v>
       </c>
-      <c r="B34" s="29" t="s">
+      <c r="B34" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="C34" s="30"/>
-      <c r="D34" s="30"/>
-      <c r="E34" s="31"/>
+      <c r="C34" s="28"/>
+      <c r="D34" s="28"/>
+      <c r="E34" s="29"/>
       <c r="F34" s="3">
         <v>24</v>
       </c>
@@ -2095,103 +2155,103 @@
       <c r="L34" s="3">
         <v>24</v>
       </c>
-      <c r="M34" s="51"/>
+      <c r="M34" s="45"/>
     </row>
     <row r="35" spans="1:13" ht="21.6" thickBot="1">
-      <c r="A35" s="37">
+      <c r="A35" s="34">
         <v>20</v>
       </c>
-      <c r="B35" s="38" t="s">
+      <c r="B35" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="C35" s="39"/>
-      <c r="D35" s="39"/>
-      <c r="E35" s="40"/>
-      <c r="F35" s="52">
-        <v>6</v>
-      </c>
-      <c r="G35" s="52">
-        <v>6</v>
-      </c>
-      <c r="H35" s="52"/>
-      <c r="I35" s="52"/>
-      <c r="J35" s="52"/>
-      <c r="K35" s="52"/>
-      <c r="L35" s="52">
-        <v>6</v>
-      </c>
-      <c r="M35" s="53"/>
+      <c r="C35" s="36"/>
+      <c r="D35" s="36"/>
+      <c r="E35" s="37"/>
+      <c r="F35" s="46">
+        <v>6</v>
+      </c>
+      <c r="G35" s="46">
+        <v>6</v>
+      </c>
+      <c r="H35" s="46"/>
+      <c r="I35" s="46"/>
+      <c r="J35" s="46"/>
+      <c r="K35" s="46"/>
+      <c r="L35" s="46">
+        <v>6</v>
+      </c>
+      <c r="M35" s="47"/>
     </row>
     <row r="36" spans="1:13" ht="21.6" thickBot="1">
-      <c r="A36" s="42" t="s">
+      <c r="A36" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B36" s="43" t="s">
+      <c r="B36" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="C36" s="43"/>
-      <c r="D36" s="43"/>
-      <c r="E36" s="43"/>
-      <c r="F36" s="44" t="s">
+      <c r="C36" s="48"/>
+      <c r="D36" s="48"/>
+      <c r="E36" s="48"/>
+      <c r="F36" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="G36" s="44" t="s">
+      <c r="G36" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="H36" s="44" t="s">
+      <c r="H36" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="I36" s="44" t="s">
-        <v>6</v>
-      </c>
-      <c r="J36" s="44" t="s">
+      <c r="I36" s="39" t="s">
+        <v>6</v>
+      </c>
+      <c r="J36" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="K36" s="44" t="s">
+      <c r="K36" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="L36" s="44" t="s">
+      <c r="L36" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="M36" s="48" t="s">
+      <c r="M36" s="42" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="37" spans="1:13">
-      <c r="A37" s="36">
+      <c r="A37" s="33">
         <v>21</v>
       </c>
-      <c r="B37" s="28" t="s">
+      <c r="B37" s="26" t="s">
         <v>64</v>
       </c>
-      <c r="C37" s="24"/>
-      <c r="D37" s="24"/>
-      <c r="E37" s="25"/>
-      <c r="F37" s="49">
-        <v>6</v>
-      </c>
-      <c r="G37" s="49">
-        <v>6</v>
-      </c>
-      <c r="H37" s="49"/>
-      <c r="I37" s="49"/>
-      <c r="J37" s="49"/>
-      <c r="K37" s="49"/>
-      <c r="L37" s="49">
-        <v>6</v>
-      </c>
-      <c r="M37" s="50"/>
+      <c r="C37" s="22"/>
+      <c r="D37" s="22"/>
+      <c r="E37" s="23"/>
+      <c r="F37" s="43">
+        <v>6</v>
+      </c>
+      <c r="G37" s="43">
+        <v>6</v>
+      </c>
+      <c r="H37" s="43"/>
+      <c r="I37" s="43"/>
+      <c r="J37" s="43"/>
+      <c r="K37" s="43"/>
+      <c r="L37" s="43">
+        <v>6</v>
+      </c>
+      <c r="M37" s="44"/>
     </row>
     <row r="38" spans="1:13">
-      <c r="A38" s="36">
+      <c r="A38" s="33">
         <v>22</v>
       </c>
-      <c r="B38" s="29" t="s">
+      <c r="B38" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="C38" s="30"/>
-      <c r="D38" s="30"/>
-      <c r="E38" s="31"/>
+      <c r="C38" s="28"/>
+      <c r="D38" s="28"/>
+      <c r="E38" s="29"/>
       <c r="F38" s="3">
         <v>6</v>
       </c>
@@ -2207,18 +2267,18 @@
       <c r="L38" s="3">
         <v>1</v>
       </c>
-      <c r="M38" s="51"/>
+      <c r="M38" s="45"/>
     </row>
     <row r="39" spans="1:13">
-      <c r="A39" s="36">
+      <c r="A39" s="33">
         <v>23</v>
       </c>
-      <c r="B39" s="17" t="s">
+      <c r="B39" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="C39" s="22"/>
-      <c r="D39" s="22"/>
-      <c r="E39" s="23"/>
+      <c r="C39" s="20"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="21"/>
       <c r="F39" s="3">
         <v>12</v>
       </c>
@@ -2234,18 +2294,17 @@
       <c r="L39" s="3">
         <v>6</v>
       </c>
-      <c r="M39" s="51"/>
+      <c r="M39" s="45"/>
     </row>
     <row r="40" spans="1:13">
-      <c r="A40" s="36"/>
-      <c r="B40" s="12" t="s">
+      <c r="A40" s="33"/>
+      <c r="B40" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="C40" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D40" s="5"/>
-      <c r="E40" s="27"/>
+      <c r="E40" s="25"/>
       <c r="F40" s="3">
         <v>12</v>
       </c>
@@ -2261,18 +2320,18 @@
       <c r="L40" s="3">
         <v>6</v>
       </c>
-      <c r="M40" s="51"/>
+      <c r="M40" s="45"/>
     </row>
     <row r="41" spans="1:13">
-      <c r="A41" s="36">
+      <c r="A41" s="33">
         <v>24</v>
       </c>
-      <c r="B41" s="29" t="s">
+      <c r="B41" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="C41" s="30"/>
-      <c r="D41" s="30"/>
-      <c r="E41" s="31"/>
+      <c r="C41" s="28"/>
+      <c r="D41" s="28"/>
+      <c r="E41" s="29"/>
       <c r="F41" s="3">
         <v>6</v>
       </c>
@@ -2288,18 +2347,18 @@
       <c r="L41" s="3">
         <v>5</v>
       </c>
-      <c r="M41" s="51"/>
+      <c r="M41" s="45"/>
     </row>
     <row r="42" spans="1:13">
-      <c r="A42" s="36">
+      <c r="A42" s="33">
         <v>25</v>
       </c>
-      <c r="B42" s="29" t="s">
+      <c r="B42" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="C42" s="30"/>
-      <c r="D42" s="30"/>
-      <c r="E42" s="31"/>
+      <c r="C42" s="28"/>
+      <c r="D42" s="28"/>
+      <c r="E42" s="29"/>
       <c r="F42" s="3">
         <v>6</v>
       </c>
@@ -2315,18 +2374,18 @@
       <c r="L42" s="3">
         <v>5</v>
       </c>
-      <c r="M42" s="51"/>
+      <c r="M42" s="45"/>
     </row>
     <row r="43" spans="1:13">
-      <c r="A43" s="36">
+      <c r="A43" s="33">
         <v>26</v>
       </c>
-      <c r="B43" s="29" t="s">
+      <c r="B43" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="C43" s="30"/>
-      <c r="D43" s="30"/>
-      <c r="E43" s="31"/>
+      <c r="C43" s="28"/>
+      <c r="D43" s="28"/>
+      <c r="E43" s="29"/>
       <c r="F43" s="3">
         <v>6</v>
       </c>
@@ -2342,18 +2401,18 @@
       <c r="L43" s="3">
         <v>1</v>
       </c>
-      <c r="M43" s="51"/>
+      <c r="M43" s="45"/>
     </row>
     <row r="44" spans="1:13">
-      <c r="A44" s="36">
+      <c r="A44" s="33">
         <v>27</v>
       </c>
-      <c r="B44" s="29" t="s">
+      <c r="B44" s="27" t="s">
         <v>46</v>
       </c>
-      <c r="C44" s="30"/>
-      <c r="D44" s="30"/>
-      <c r="E44" s="31"/>
+      <c r="C44" s="28"/>
+      <c r="D44" s="28"/>
+      <c r="E44" s="29"/>
       <c r="F44" s="3">
         <v>60</v>
       </c>
@@ -2369,18 +2428,18 @@
       <c r="L44" s="3">
         <v>40</v>
       </c>
-      <c r="M44" s="51"/>
+      <c r="M44" s="45"/>
     </row>
     <row r="45" spans="1:13">
-      <c r="A45" s="36">
+      <c r="A45" s="33">
         <v>28</v>
       </c>
-      <c r="B45" s="29" t="s">
+      <c r="B45" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="C45" s="30"/>
-      <c r="D45" s="30"/>
-      <c r="E45" s="31"/>
+      <c r="C45" s="28"/>
+      <c r="D45" s="28"/>
+      <c r="E45" s="29"/>
       <c r="F45" s="3">
         <v>6</v>
       </c>
@@ -2396,18 +2455,18 @@
       <c r="L45" s="3">
         <v>5</v>
       </c>
-      <c r="M45" s="51"/>
+      <c r="M45" s="45"/>
     </row>
     <row r="46" spans="1:13">
-      <c r="A46" s="36">
+      <c r="A46" s="33">
         <v>29</v>
       </c>
-      <c r="B46" s="29" t="s">
+      <c r="B46" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="C46" s="30"/>
-      <c r="D46" s="30"/>
-      <c r="E46" s="31"/>
+      <c r="C46" s="28"/>
+      <c r="D46" s="28"/>
+      <c r="E46" s="29"/>
       <c r="F46" s="3">
         <v>6</v>
       </c>
@@ -2423,18 +2482,18 @@
       <c r="L46" s="3">
         <v>4</v>
       </c>
-      <c r="M46" s="51"/>
+      <c r="M46" s="45"/>
     </row>
     <row r="47" spans="1:13">
-      <c r="A47" s="36">
+      <c r="A47" s="33">
         <v>30</v>
       </c>
-      <c r="B47" s="29" t="s">
+      <c r="B47" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="C47" s="30"/>
-      <c r="D47" s="30"/>
-      <c r="E47" s="31"/>
+      <c r="C47" s="28"/>
+      <c r="D47" s="28"/>
+      <c r="E47" s="29"/>
       <c r="F47" s="3">
         <v>6</v>
       </c>
@@ -2450,18 +2509,18 @@
       <c r="L47" s="3">
         <v>5</v>
       </c>
-      <c r="M47" s="51"/>
+      <c r="M47" s="45"/>
     </row>
     <row r="48" spans="1:13">
-      <c r="A48" s="36">
+      <c r="A48" s="33">
         <v>31</v>
       </c>
-      <c r="B48" s="29" t="s">
+      <c r="B48" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="C48" s="30"/>
-      <c r="D48" s="30"/>
-      <c r="E48" s="31"/>
+      <c r="C48" s="28"/>
+      <c r="D48" s="28"/>
+      <c r="E48" s="29"/>
       <c r="F48" s="3">
         <v>36</v>
       </c>
@@ -2477,18 +2536,18 @@
       <c r="L48" s="3">
         <v>24</v>
       </c>
-      <c r="M48" s="51"/>
+      <c r="M48" s="45"/>
     </row>
     <row r="49" spans="1:13">
-      <c r="A49" s="36">
+      <c r="A49" s="33">
         <v>32</v>
       </c>
-      <c r="B49" s="29" t="s">
+      <c r="B49" s="27" t="s">
         <v>51</v>
       </c>
-      <c r="C49" s="30"/>
-      <c r="D49" s="30"/>
-      <c r="E49" s="31"/>
+      <c r="C49" s="28"/>
+      <c r="D49" s="28"/>
+      <c r="E49" s="29"/>
       <c r="F49" s="3">
         <v>6</v>
       </c>
@@ -2504,18 +2563,18 @@
       <c r="L49" s="3">
         <v>1</v>
       </c>
-      <c r="M49" s="51"/>
+      <c r="M49" s="45"/>
     </row>
     <row r="50" spans="1:13">
-      <c r="A50" s="36">
+      <c r="A50" s="33">
         <v>33</v>
       </c>
-      <c r="B50" s="29" t="s">
+      <c r="B50" s="27" t="s">
         <v>52</v>
       </c>
-      <c r="C50" s="30"/>
-      <c r="D50" s="30"/>
-      <c r="E50" s="31"/>
+      <c r="C50" s="28"/>
+      <c r="D50" s="28"/>
+      <c r="E50" s="29"/>
       <c r="F50" s="3">
         <v>6</v>
       </c>
@@ -2531,18 +2590,18 @@
       <c r="L50" s="3">
         <v>0</v>
       </c>
-      <c r="M50" s="51"/>
+      <c r="M50" s="45"/>
     </row>
     <row r="51" spans="1:13">
-      <c r="A51" s="36">
+      <c r="A51" s="33">
         <v>34</v>
       </c>
-      <c r="B51" s="29" t="s">
+      <c r="B51" s="27" t="s">
         <v>53</v>
       </c>
-      <c r="C51" s="30"/>
-      <c r="D51" s="30"/>
-      <c r="E51" s="31"/>
+      <c r="C51" s="28"/>
+      <c r="D51" s="28"/>
+      <c r="E51" s="29"/>
       <c r="F51" s="3">
         <v>6</v>
       </c>
@@ -2558,18 +2617,18 @@
       <c r="L51" s="3">
         <v>4</v>
       </c>
-      <c r="M51" s="51"/>
+      <c r="M51" s="45"/>
     </row>
     <row r="52" spans="1:13">
-      <c r="A52" s="36">
+      <c r="A52" s="33">
         <v>35</v>
       </c>
-      <c r="B52" s="29" t="s">
+      <c r="B52" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="C52" s="30"/>
-      <c r="D52" s="30"/>
-      <c r="E52" s="31"/>
+      <c r="C52" s="28"/>
+      <c r="D52" s="28"/>
+      <c r="E52" s="29"/>
       <c r="F52" s="3">
         <v>60</v>
       </c>
@@ -2585,18 +2644,18 @@
       <c r="L52" s="3">
         <v>40</v>
       </c>
-      <c r="M52" s="51"/>
+      <c r="M52" s="45"/>
     </row>
     <row r="53" spans="1:13">
-      <c r="A53" s="36">
+      <c r="A53" s="33">
         <v>36</v>
       </c>
-      <c r="B53" s="29" t="s">
+      <c r="B53" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="C53" s="30"/>
-      <c r="D53" s="30"/>
-      <c r="E53" s="31"/>
+      <c r="C53" s="28"/>
+      <c r="D53" s="28"/>
+      <c r="E53" s="29"/>
       <c r="F53" s="3">
         <v>6</v>
       </c>
@@ -2612,18 +2671,18 @@
       <c r="L53" s="3">
         <v>0</v>
       </c>
-      <c r="M53" s="51"/>
+      <c r="M53" s="45"/>
     </row>
     <row r="54" spans="1:13">
-      <c r="A54" s="36">
+      <c r="A54" s="33">
         <v>37</v>
       </c>
-      <c r="B54" s="29" t="s">
+      <c r="B54" s="27" t="s">
         <v>56</v>
       </c>
-      <c r="C54" s="30"/>
-      <c r="D54" s="30"/>
-      <c r="E54" s="31"/>
+      <c r="C54" s="28"/>
+      <c r="D54" s="28"/>
+      <c r="E54" s="29"/>
       <c r="F54" s="3">
         <v>6</v>
       </c>
@@ -2637,18 +2696,18 @@
       <c r="L54" s="3">
         <v>6</v>
       </c>
-      <c r="M54" s="51"/>
+      <c r="M54" s="45"/>
     </row>
     <row r="55" spans="1:13">
-      <c r="A55" s="36">
+      <c r="A55" s="33">
         <v>38</v>
       </c>
-      <c r="B55" s="29" t="s">
+      <c r="B55" s="27" t="s">
         <v>57</v>
       </c>
-      <c r="C55" s="30"/>
-      <c r="D55" s="30"/>
-      <c r="E55" s="31"/>
+      <c r="C55" s="28"/>
+      <c r="D55" s="28"/>
+      <c r="E55" s="29"/>
       <c r="F55" s="3">
         <v>18</v>
       </c>
@@ -2664,18 +2723,18 @@
       <c r="L55" s="3">
         <v>14</v>
       </c>
-      <c r="M55" s="51"/>
+      <c r="M55" s="45"/>
     </row>
     <row r="56" spans="1:13">
-      <c r="A56" s="36">
+      <c r="A56" s="33">
         <v>39</v>
       </c>
-      <c r="B56" s="29" t="s">
+      <c r="B56" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="C56" s="30"/>
-      <c r="D56" s="30"/>
-      <c r="E56" s="31"/>
+      <c r="C56" s="28"/>
+      <c r="D56" s="28"/>
+      <c r="E56" s="29"/>
       <c r="F56" s="3">
         <v>6</v>
       </c>
@@ -2689,18 +2748,18 @@
       <c r="L56" s="3">
         <v>6</v>
       </c>
-      <c r="M56" s="51"/>
+      <c r="M56" s="45"/>
     </row>
     <row r="57" spans="1:13">
-      <c r="A57" s="36">
+      <c r="A57" s="33">
         <v>40</v>
       </c>
-      <c r="B57" s="29" t="s">
+      <c r="B57" s="27" t="s">
         <v>109</v>
       </c>
-      <c r="C57" s="30"/>
-      <c r="D57" s="30"/>
-      <c r="E57" s="31"/>
+      <c r="C57" s="28"/>
+      <c r="D57" s="28"/>
+      <c r="E57" s="29"/>
       <c r="F57" s="3">
         <v>240</v>
       </c>
@@ -2716,18 +2775,16 @@
       <c r="L57" s="3">
         <v>80</v>
       </c>
-      <c r="M57" s="51"/>
+      <c r="M57" s="45"/>
     </row>
     <row r="58" spans="1:13">
-      <c r="A58" s="36">
+      <c r="A58" s="33">
         <v>41</v>
       </c>
-      <c r="B58" s="26" t="s">
+      <c r="B58" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="C58" s="5"/>
-      <c r="D58" s="5"/>
-      <c r="E58" s="27"/>
+      <c r="E58" s="25"/>
       <c r="F58" s="3">
         <v>6</v>
       </c>
@@ -2741,18 +2798,17 @@
       <c r="L58" s="3">
         <v>6</v>
       </c>
-      <c r="M58" s="51"/>
+      <c r="M58" s="45"/>
     </row>
     <row r="59" spans="1:13">
-      <c r="A59" s="36"/>
-      <c r="B59" s="12" t="s">
+      <c r="A59" s="33"/>
+      <c r="B59" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C59" s="5" t="s">
+      <c r="C59" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D59" s="5"/>
-      <c r="E59" s="27"/>
+      <c r="E59" s="25"/>
       <c r="F59" s="3">
         <v>6</v>
       </c>
@@ -2766,18 +2822,18 @@
       <c r="L59" s="3">
         <v>6</v>
       </c>
-      <c r="M59" s="51"/>
+      <c r="M59" s="45"/>
     </row>
     <row r="60" spans="1:13">
-      <c r="A60" s="36">
+      <c r="A60" s="33">
         <v>42</v>
       </c>
-      <c r="B60" s="29" t="s">
+      <c r="B60" s="27" t="s">
         <v>89</v>
       </c>
-      <c r="C60" s="32"/>
-      <c r="D60" s="30"/>
-      <c r="E60" s="31"/>
+      <c r="C60" s="30"/>
+      <c r="D60" s="28"/>
+      <c r="E60" s="29"/>
       <c r="F60" s="3">
         <v>18</v>
       </c>
@@ -2791,18 +2847,18 @@
       <c r="L60" s="3">
         <v>18</v>
       </c>
-      <c r="M60" s="51"/>
+      <c r="M60" s="45"/>
     </row>
     <row r="61" spans="1:13">
-      <c r="A61" s="36">
+      <c r="A61" s="33">
         <v>43</v>
       </c>
-      <c r="B61" s="29" t="s">
+      <c r="B61" s="27" t="s">
         <v>96</v>
       </c>
-      <c r="C61" s="30"/>
-      <c r="D61" s="30"/>
-      <c r="E61" s="31"/>
+      <c r="C61" s="28"/>
+      <c r="D61" s="28"/>
+      <c r="E61" s="29"/>
       <c r="F61" s="3">
         <v>9</v>
       </c>
@@ -2816,18 +2872,18 @@
       <c r="L61" s="3">
         <v>9</v>
       </c>
-      <c r="M61" s="51"/>
+      <c r="M61" s="45"/>
     </row>
     <row r="62" spans="1:13">
-      <c r="A62" s="36">
+      <c r="A62" s="33">
         <v>42</v>
       </c>
-      <c r="B62" s="29" t="s">
+      <c r="B62" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="C62" s="30"/>
-      <c r="D62" s="30"/>
-      <c r="E62" s="31"/>
+      <c r="C62" s="28"/>
+      <c r="D62" s="28"/>
+      <c r="E62" s="29"/>
       <c r="F62" s="3">
         <v>6</v>
       </c>
@@ -2843,106 +2899,106 @@
       <c r="L62" s="3">
         <v>7</v>
       </c>
-      <c r="M62" s="51"/>
+      <c r="M62" s="45"/>
     </row>
     <row r="63" spans="1:13" ht="21.6" thickBot="1">
-      <c r="A63" s="37">
+      <c r="A63" s="34">
         <v>43</v>
       </c>
-      <c r="B63" s="38" t="s">
+      <c r="B63" s="35" t="s">
         <v>98</v>
       </c>
-      <c r="C63" s="39"/>
-      <c r="D63" s="39"/>
-      <c r="E63" s="40"/>
-      <c r="F63" s="52">
+      <c r="C63" s="36"/>
+      <c r="D63" s="36"/>
+      <c r="E63" s="37"/>
+      <c r="F63" s="46">
         <v>5</v>
       </c>
-      <c r="G63" s="52">
+      <c r="G63" s="46">
         <v>5</v>
       </c>
-      <c r="H63" s="52"/>
-      <c r="I63" s="52"/>
-      <c r="J63" s="52"/>
-      <c r="K63" s="52"/>
-      <c r="L63" s="52">
+      <c r="H63" s="46"/>
+      <c r="I63" s="46"/>
+      <c r="J63" s="46"/>
+      <c r="K63" s="46"/>
+      <c r="L63" s="46">
         <v>5</v>
       </c>
-      <c r="M63" s="53"/>
+      <c r="M63" s="47"/>
     </row>
     <row r="70" spans="1:13" ht="21.6" thickBot="1"/>
     <row r="71" spans="1:13" ht="21.6" thickBot="1">
-      <c r="A71" s="42" t="s">
+      <c r="A71" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B71" s="43" t="s">
+      <c r="B71" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="C71" s="43"/>
-      <c r="D71" s="43"/>
-      <c r="E71" s="43"/>
-      <c r="F71" s="44" t="s">
+      <c r="C71" s="48"/>
+      <c r="D71" s="48"/>
+      <c r="E71" s="48"/>
+      <c r="F71" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="G71" s="44" t="s">
+      <c r="G71" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="H71" s="44" t="s">
+      <c r="H71" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="I71" s="44" t="s">
-        <v>6</v>
-      </c>
-      <c r="J71" s="44" t="s">
+      <c r="I71" s="39" t="s">
+        <v>6</v>
+      </c>
+      <c r="J71" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="K71" s="44" t="s">
+      <c r="K71" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="L71" s="44" t="s">
+      <c r="L71" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="M71" s="48" t="s">
+      <c r="M71" s="42" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="72" spans="1:13">
-      <c r="A72" s="36">
+      <c r="A72" s="50">
         <v>1</v>
       </c>
-      <c r="B72" s="28" t="s">
+      <c r="B72" s="51" t="s">
         <v>65</v>
       </c>
-      <c r="C72" s="24"/>
-      <c r="D72" s="24"/>
-      <c r="E72" s="25"/>
-      <c r="F72" s="49">
-        <v>6</v>
-      </c>
-      <c r="G72" s="49">
+      <c r="C72" s="52"/>
+      <c r="D72" s="52"/>
+      <c r="E72" s="53"/>
+      <c r="F72" s="54">
+        <v>6</v>
+      </c>
+      <c r="G72" s="54">
         <v>5</v>
       </c>
-      <c r="H72" s="49">
+      <c r="H72" s="54">
         <v>1</v>
       </c>
-      <c r="I72" s="49"/>
-      <c r="J72" s="49"/>
-      <c r="K72" s="49"/>
-      <c r="L72" s="49">
+      <c r="I72" s="54"/>
+      <c r="J72" s="54"/>
+      <c r="K72" s="54"/>
+      <c r="L72" s="54">
         <v>5</v>
       </c>
-      <c r="M72" s="50"/>
+      <c r="M72" s="55"/>
     </row>
     <row r="73" spans="1:13">
-      <c r="A73" s="36">
+      <c r="A73" s="33">
         <v>2</v>
       </c>
-      <c r="B73" s="26" t="s">
+      <c r="B73" s="24" t="s">
         <v>66</v>
       </c>
-      <c r="C73" s="5"/>
-      <c r="D73" s="5"/>
-      <c r="E73" s="27"/>
+      <c r="C73" s="56"/>
+      <c r="D73" s="56"/>
+      <c r="E73" s="25"/>
       <c r="F73" s="3">
         <v>6</v>
       </c>
@@ -2958,18 +3014,18 @@
       <c r="L73" s="3">
         <v>5</v>
       </c>
-      <c r="M73" s="51"/>
+      <c r="M73" s="45"/>
     </row>
     <row r="74" spans="1:13">
-      <c r="A74" s="36">
+      <c r="A74" s="33">
         <v>3</v>
       </c>
-      <c r="B74" s="17" t="s">
+      <c r="B74" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="C74" s="22"/>
-      <c r="D74" s="22"/>
-      <c r="E74" s="23"/>
+      <c r="C74" s="20"/>
+      <c r="D74" s="20"/>
+      <c r="E74" s="21"/>
       <c r="F74" s="3"/>
       <c r="G74" s="3"/>
       <c r="H74" s="3"/>
@@ -2977,18 +3033,18 @@
       <c r="J74" s="3"/>
       <c r="K74" s="3"/>
       <c r="L74" s="3"/>
-      <c r="M74" s="51"/>
+      <c r="M74" s="45"/>
     </row>
     <row r="75" spans="1:13">
-      <c r="A75" s="36"/>
-      <c r="B75" s="12" t="s">
+      <c r="A75" s="33"/>
+      <c r="B75" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C75" s="5" t="s">
+      <c r="C75" s="56" t="s">
         <v>70</v>
       </c>
-      <c r="D75" s="5"/>
-      <c r="E75" s="27"/>
+      <c r="D75" s="56"/>
+      <c r="E75" s="25"/>
       <c r="F75" s="3">
         <v>6</v>
       </c>
@@ -3006,18 +3062,18 @@
         <f t="shared" ref="L75:L77" si="1">G75</f>
         <v>6</v>
       </c>
-      <c r="M75" s="51"/>
+      <c r="M75" s="45"/>
     </row>
     <row r="76" spans="1:13">
-      <c r="A76" s="36"/>
-      <c r="B76" s="12" t="s">
+      <c r="A76" s="33"/>
+      <c r="B76" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C76" s="5" t="s">
+      <c r="C76" s="56" t="s">
         <v>69</v>
       </c>
-      <c r="D76" s="5"/>
-      <c r="E76" s="27"/>
+      <c r="D76" s="56"/>
+      <c r="E76" s="25"/>
       <c r="F76" s="3">
         <v>6</v>
       </c>
@@ -3035,18 +3091,18 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="M76" s="51"/>
+      <c r="M76" s="45"/>
     </row>
     <row r="77" spans="1:13">
-      <c r="A77" s="36"/>
-      <c r="B77" s="14" t="s">
+      <c r="A77" s="33"/>
+      <c r="B77" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C77" s="24" t="s">
+      <c r="C77" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="D77" s="24"/>
-      <c r="E77" s="25"/>
+      <c r="D77" s="22"/>
+      <c r="E77" s="23"/>
       <c r="F77" s="3">
         <v>6</v>
       </c>
@@ -3064,18 +3120,18 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="M77" s="51"/>
+      <c r="M77" s="45"/>
     </row>
     <row r="78" spans="1:13">
-      <c r="A78" s="36">
+      <c r="A78" s="33">
         <v>4</v>
       </c>
-      <c r="B78" s="26" t="s">
+      <c r="B78" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="C78" s="5"/>
-      <c r="D78" s="5"/>
-      <c r="E78" s="27"/>
+      <c r="C78" s="56"/>
+      <c r="D78" s="56"/>
+      <c r="E78" s="25"/>
       <c r="F78" s="3">
         <v>6</v>
       </c>
@@ -3093,18 +3149,18 @@
         <f t="shared" ref="L78:L105" si="3">G78</f>
         <v>4</v>
       </c>
-      <c r="M78" s="51"/>
+      <c r="M78" s="45"/>
     </row>
     <row r="79" spans="1:13">
-      <c r="A79" s="36">
+      <c r="A79" s="33">
         <v>5</v>
       </c>
-      <c r="B79" s="17" t="s">
+      <c r="B79" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="C79" s="22"/>
-      <c r="D79" s="22"/>
-      <c r="E79" s="23"/>
+      <c r="C79" s="20"/>
+      <c r="D79" s="20"/>
+      <c r="E79" s="21"/>
       <c r="F79" s="3"/>
       <c r="G79" s="3"/>
       <c r="H79" s="3"/>
@@ -3112,18 +3168,18 @@
       <c r="J79" s="3"/>
       <c r="K79" s="3"/>
       <c r="L79" s="3"/>
-      <c r="M79" s="51"/>
+      <c r="M79" s="45"/>
     </row>
     <row r="80" spans="1:13">
-      <c r="A80" s="36"/>
-      <c r="B80" s="12" t="s">
+      <c r="A80" s="33"/>
+      <c r="B80" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C80" s="5" t="s">
+      <c r="C80" s="56" t="s">
         <v>70</v>
       </c>
-      <c r="D80" s="5"/>
-      <c r="E80" s="27"/>
+      <c r="D80" s="56"/>
+      <c r="E80" s="25"/>
       <c r="F80" s="3">
         <v>6</v>
       </c>
@@ -3141,18 +3197,18 @@
         <f t="shared" ref="L80:L81" si="5">G80</f>
         <v>6</v>
       </c>
-      <c r="M80" s="51"/>
+      <c r="M80" s="45"/>
     </row>
     <row r="81" spans="1:13">
-      <c r="A81" s="36"/>
-      <c r="B81" s="14" t="s">
+      <c r="A81" s="33"/>
+      <c r="B81" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C81" s="24" t="s">
+      <c r="C81" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="D81" s="24"/>
-      <c r="E81" s="25"/>
+      <c r="D81" s="22"/>
+      <c r="E81" s="23"/>
       <c r="F81" s="3">
         <v>6</v>
       </c>
@@ -3170,18 +3226,18 @@
         <f t="shared" si="5"/>
         <v>5</v>
       </c>
-      <c r="M81" s="51"/>
+      <c r="M81" s="45"/>
     </row>
     <row r="82" spans="1:13">
-      <c r="A82" s="36">
-        <v>6</v>
-      </c>
-      <c r="B82" s="26" t="s">
+      <c r="A82" s="33">
+        <v>6</v>
+      </c>
+      <c r="B82" s="24" t="s">
         <v>74</v>
       </c>
-      <c r="C82" s="5"/>
-      <c r="D82" s="5"/>
-      <c r="E82" s="27"/>
+      <c r="C82" s="56"/>
+      <c r="D82" s="56"/>
+      <c r="E82" s="25"/>
       <c r="F82" s="3">
         <v>6</v>
       </c>
@@ -3199,18 +3255,18 @@
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="M82" s="51"/>
+      <c r="M82" s="45"/>
     </row>
     <row r="83" spans="1:13">
-      <c r="A83" s="36">
+      <c r="A83" s="33">
         <v>7</v>
       </c>
-      <c r="B83" s="29" t="s">
+      <c r="B83" s="27" t="s">
         <v>75</v>
       </c>
-      <c r="C83" s="30"/>
-      <c r="D83" s="30"/>
-      <c r="E83" s="31"/>
+      <c r="C83" s="28"/>
+      <c r="D83" s="28"/>
+      <c r="E83" s="29"/>
       <c r="F83" s="3">
         <v>6</v>
       </c>
@@ -3228,18 +3284,18 @@
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="M83" s="51"/>
+      <c r="M83" s="45"/>
     </row>
     <row r="84" spans="1:13">
-      <c r="A84" s="36">
+      <c r="A84" s="33">
         <v>8</v>
       </c>
-      <c r="B84" s="29" t="s">
+      <c r="B84" s="27" t="s">
         <v>76</v>
       </c>
-      <c r="C84" s="30"/>
-      <c r="D84" s="30"/>
-      <c r="E84" s="31"/>
+      <c r="C84" s="28"/>
+      <c r="D84" s="28"/>
+      <c r="E84" s="29"/>
       <c r="F84" s="3">
         <v>6</v>
       </c>
@@ -3257,18 +3313,18 @@
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="M84" s="51"/>
+      <c r="M84" s="45"/>
     </row>
     <row r="85" spans="1:13">
-      <c r="A85" s="36">
+      <c r="A85" s="33">
         <v>9</v>
       </c>
-      <c r="B85" s="29" t="s">
+      <c r="B85" s="27" t="s">
         <v>77</v>
       </c>
-      <c r="C85" s="30"/>
-      <c r="D85" s="30"/>
-      <c r="E85" s="31"/>
+      <c r="C85" s="28"/>
+      <c r="D85" s="28"/>
+      <c r="E85" s="29"/>
       <c r="F85" s="3">
         <v>6</v>
       </c>
@@ -3286,18 +3342,18 @@
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="M85" s="51"/>
+      <c r="M85" s="45"/>
     </row>
     <row r="86" spans="1:13">
-      <c r="A86" s="36">
+      <c r="A86" s="33">
         <v>10</v>
       </c>
-      <c r="B86" s="29" t="s">
+      <c r="B86" s="27" t="s">
         <v>78</v>
       </c>
-      <c r="C86" s="30"/>
-      <c r="D86" s="30"/>
-      <c r="E86" s="31"/>
+      <c r="C86" s="28"/>
+      <c r="D86" s="28"/>
+      <c r="E86" s="29"/>
       <c r="F86" s="3">
         <v>6</v>
       </c>
@@ -3315,18 +3371,18 @@
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="M86" s="51"/>
+      <c r="M86" s="45"/>
     </row>
     <row r="87" spans="1:13">
-      <c r="A87" s="36">
+      <c r="A87" s="33">
         <v>11</v>
       </c>
-      <c r="B87" s="29" t="s">
+      <c r="B87" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="C87" s="30"/>
-      <c r="D87" s="30"/>
-      <c r="E87" s="31"/>
+      <c r="C87" s="28"/>
+      <c r="D87" s="28"/>
+      <c r="E87" s="29"/>
       <c r="F87" s="3">
         <v>6</v>
       </c>
@@ -3344,18 +3400,18 @@
         <f t="shared" ref="L87:L89" si="7">G87</f>
         <v>6</v>
       </c>
-      <c r="M87" s="51"/>
+      <c r="M87" s="45"/>
     </row>
     <row r="88" spans="1:13">
-      <c r="A88" s="36">
+      <c r="A88" s="33">
         <v>12</v>
       </c>
-      <c r="B88" s="29" t="s">
+      <c r="B88" s="27" t="s">
         <v>80</v>
       </c>
-      <c r="C88" s="30"/>
-      <c r="D88" s="30"/>
-      <c r="E88" s="31"/>
+      <c r="C88" s="28"/>
+      <c r="D88" s="28"/>
+      <c r="E88" s="29"/>
       <c r="F88" s="3">
         <v>6</v>
       </c>
@@ -3373,18 +3429,18 @@
         <f t="shared" si="7"/>
         <v>6</v>
       </c>
-      <c r="M88" s="51"/>
+      <c r="M88" s="45"/>
     </row>
     <row r="89" spans="1:13">
-      <c r="A89" s="36">
+      <c r="A89" s="33">
         <v>13</v>
       </c>
-      <c r="B89" s="26" t="s">
+      <c r="B89" s="24" t="s">
         <v>81</v>
       </c>
-      <c r="C89" s="5"/>
-      <c r="D89" s="5"/>
-      <c r="E89" s="27"/>
+      <c r="C89" s="56"/>
+      <c r="D89" s="56"/>
+      <c r="E89" s="25"/>
       <c r="F89" s="3">
         <v>6</v>
       </c>
@@ -3402,18 +3458,18 @@
         <f t="shared" si="7"/>
         <v>6</v>
       </c>
-      <c r="M89" s="51"/>
+      <c r="M89" s="45"/>
     </row>
     <row r="90" spans="1:13">
-      <c r="A90" s="36">
+      <c r="A90" s="33">
         <v>14</v>
       </c>
-      <c r="B90" s="17" t="s">
+      <c r="B90" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="C90" s="22"/>
-      <c r="D90" s="22"/>
-      <c r="E90" s="23"/>
+      <c r="C90" s="20"/>
+      <c r="D90" s="20"/>
+      <c r="E90" s="21"/>
       <c r="F90" s="3"/>
       <c r="G90" s="3"/>
       <c r="H90" s="3"/>
@@ -3421,18 +3477,18 @@
       <c r="J90" s="3"/>
       <c r="K90" s="3"/>
       <c r="L90" s="3"/>
-      <c r="M90" s="51"/>
+      <c r="M90" s="45"/>
     </row>
     <row r="91" spans="1:13">
-      <c r="A91" s="36"/>
-      <c r="B91" s="12" t="s">
+      <c r="A91" s="33"/>
+      <c r="B91" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C91" s="5" t="s">
+      <c r="C91" s="56" t="s">
         <v>83</v>
       </c>
-      <c r="D91" s="5"/>
-      <c r="E91" s="27"/>
+      <c r="D91" s="56"/>
+      <c r="E91" s="25"/>
       <c r="F91" s="3">
         <v>6</v>
       </c>
@@ -3450,18 +3506,18 @@
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="M91" s="51"/>
+      <c r="M91" s="45"/>
     </row>
     <row r="92" spans="1:13">
-      <c r="A92" s="36"/>
-      <c r="B92" s="12" t="s">
+      <c r="A92" s="33"/>
+      <c r="B92" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C92" s="5" t="s">
+      <c r="C92" s="56" t="s">
         <v>84</v>
       </c>
-      <c r="D92" s="5"/>
-      <c r="E92" s="27"/>
+      <c r="D92" s="56"/>
+      <c r="E92" s="25"/>
       <c r="F92" s="3">
         <v>6</v>
       </c>
@@ -3479,18 +3535,18 @@
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="M92" s="51"/>
+      <c r="M92" s="45"/>
     </row>
     <row r="93" spans="1:13">
-      <c r="A93" s="36">
+      <c r="A93" s="33">
         <v>15</v>
       </c>
-      <c r="B93" s="29" t="s">
+      <c r="B93" s="27" t="s">
         <v>85</v>
       </c>
-      <c r="C93" s="30"/>
-      <c r="D93" s="30"/>
-      <c r="E93" s="31"/>
+      <c r="C93" s="28"/>
+      <c r="D93" s="28"/>
+      <c r="E93" s="29"/>
       <c r="F93" s="3">
         <v>6</v>
       </c>
@@ -3508,18 +3564,18 @@
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="M93" s="51"/>
+      <c r="M93" s="45"/>
     </row>
     <row r="94" spans="1:13">
-      <c r="A94" s="36">
+      <c r="A94" s="33">
         <v>16</v>
       </c>
-      <c r="B94" s="29" t="s">
+      <c r="B94" s="27" t="s">
         <v>86</v>
       </c>
-      <c r="C94" s="30"/>
-      <c r="D94" s="30"/>
-      <c r="E94" s="31"/>
+      <c r="C94" s="28"/>
+      <c r="D94" s="28"/>
+      <c r="E94" s="29"/>
       <c r="F94" s="3">
         <v>6</v>
       </c>
@@ -3537,18 +3593,18 @@
         <f t="shared" ref="L94:L95" si="9">G94</f>
         <v>6</v>
       </c>
-      <c r="M94" s="51"/>
+      <c r="M94" s="45"/>
     </row>
     <row r="95" spans="1:13">
-      <c r="A95" s="36">
+      <c r="A95" s="33">
         <v>17</v>
       </c>
-      <c r="B95" s="29" t="s">
+      <c r="B95" s="27" t="s">
         <v>87</v>
       </c>
-      <c r="C95" s="30"/>
-      <c r="D95" s="30"/>
-      <c r="E95" s="31"/>
+      <c r="C95" s="28"/>
+      <c r="D95" s="28"/>
+      <c r="E95" s="29"/>
       <c r="F95" s="3">
         <v>6</v>
       </c>
@@ -3566,18 +3622,18 @@
         <f t="shared" si="9"/>
         <v>6</v>
       </c>
-      <c r="M95" s="51"/>
+      <c r="M95" s="45"/>
     </row>
     <row r="96" spans="1:13">
-      <c r="A96" s="36">
+      <c r="A96" s="33">
         <v>18</v>
       </c>
-      <c r="B96" s="29" t="s">
+      <c r="B96" s="27" t="s">
         <v>88</v>
       </c>
-      <c r="C96" s="30"/>
-      <c r="D96" s="30"/>
-      <c r="E96" s="31"/>
+      <c r="C96" s="28"/>
+      <c r="D96" s="28"/>
+      <c r="E96" s="29"/>
       <c r="F96" s="3">
         <v>6</v>
       </c>
@@ -3595,18 +3651,18 @@
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="M96" s="51"/>
+      <c r="M96" s="45"/>
     </row>
     <row r="97" spans="1:13">
-      <c r="A97" s="36">
+      <c r="A97" s="33">
         <v>19</v>
       </c>
-      <c r="B97" s="29" t="s">
+      <c r="B97" s="27" t="s">
         <v>90</v>
       </c>
-      <c r="C97" s="30"/>
-      <c r="D97" s="30"/>
-      <c r="E97" s="31"/>
+      <c r="C97" s="28"/>
+      <c r="D97" s="28"/>
+      <c r="E97" s="29"/>
       <c r="F97" s="3">
         <v>6</v>
       </c>
@@ -3624,18 +3680,18 @@
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="M97" s="51"/>
+      <c r="M97" s="45"/>
     </row>
     <row r="98" spans="1:13">
-      <c r="A98" s="36">
+      <c r="A98" s="33">
         <v>20</v>
       </c>
-      <c r="B98" s="26" t="s">
+      <c r="B98" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="C98" s="5"/>
-      <c r="D98" s="5"/>
-      <c r="E98" s="27"/>
+      <c r="C98" s="56"/>
+      <c r="D98" s="56"/>
+      <c r="E98" s="25"/>
       <c r="F98" s="3">
         <v>6</v>
       </c>
@@ -3653,43 +3709,37 @@
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="M98" s="51"/>
+      <c r="M98" s="45"/>
     </row>
     <row r="99" spans="1:13">
-      <c r="A99" s="36">
+      <c r="A99" s="33">
         <v>21</v>
       </c>
-      <c r="B99" s="17" t="s">
+      <c r="B99" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="C99" s="22"/>
-      <c r="D99" s="22"/>
-      <c r="E99" s="23"/>
+      <c r="C99" s="20"/>
+      <c r="D99" s="20"/>
+      <c r="E99" s="21"/>
       <c r="F99" s="3"/>
       <c r="G99" s="3"/>
-      <c r="H99" s="3">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="H99" s="3"/>
       <c r="I99" s="3"/>
       <c r="J99" s="3"/>
       <c r="K99" s="3"/>
-      <c r="L99" s="3">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="M99" s="51"/>
+      <c r="L99" s="3"/>
+      <c r="M99" s="45"/>
     </row>
     <row r="100" spans="1:13">
-      <c r="A100" s="36"/>
-      <c r="B100" s="12" t="s">
+      <c r="A100" s="33"/>
+      <c r="B100" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C100" s="5" t="s">
+      <c r="C100" s="56" t="s">
         <v>93</v>
       </c>
-      <c r="D100" s="5"/>
-      <c r="E100" s="27"/>
+      <c r="D100" s="56"/>
+      <c r="E100" s="25"/>
       <c r="F100" s="3">
         <v>6</v>
       </c>
@@ -3707,18 +3757,18 @@
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="M100" s="51"/>
+      <c r="M100" s="45"/>
     </row>
     <row r="101" spans="1:13">
-      <c r="A101" s="36"/>
-      <c r="B101" s="14" t="s">
+      <c r="A101" s="33"/>
+      <c r="B101" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C101" s="24" t="s">
+      <c r="C101" s="22" t="s">
         <v>94</v>
       </c>
-      <c r="D101" s="24"/>
-      <c r="E101" s="25"/>
+      <c r="D101" s="22"/>
+      <c r="E101" s="23"/>
       <c r="F101" s="3">
         <v>6</v>
       </c>
@@ -3736,18 +3786,18 @@
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="M101" s="51"/>
+      <c r="M101" s="45"/>
     </row>
     <row r="102" spans="1:13">
-      <c r="A102" s="36">
+      <c r="A102" s="33">
         <v>22</v>
       </c>
-      <c r="B102" s="26" t="s">
+      <c r="B102" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="C102" s="5"/>
-      <c r="D102" s="5"/>
-      <c r="E102" s="27"/>
+      <c r="C102" s="56"/>
+      <c r="D102" s="56"/>
+      <c r="E102" s="25"/>
       <c r="F102" s="3">
         <v>6</v>
       </c>
@@ -3765,18 +3815,18 @@
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="M102" s="51"/>
+      <c r="M102" s="45"/>
     </row>
     <row r="103" spans="1:13">
-      <c r="A103" s="36">
+      <c r="A103" s="33">
         <v>23</v>
       </c>
-      <c r="B103" s="29" t="s">
+      <c r="B103" s="27" t="s">
         <v>99</v>
       </c>
-      <c r="C103" s="30"/>
-      <c r="D103" s="30"/>
-      <c r="E103" s="31"/>
+      <c r="C103" s="28"/>
+      <c r="D103" s="28"/>
+      <c r="E103" s="29"/>
       <c r="F103" s="3">
         <v>6</v>
       </c>
@@ -3794,18 +3844,18 @@
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="M103" s="51"/>
+      <c r="M103" s="45"/>
     </row>
     <row r="104" spans="1:13">
-      <c r="A104" s="36">
+      <c r="A104" s="33">
         <v>24</v>
       </c>
-      <c r="B104" s="29" t="s">
+      <c r="B104" s="27" t="s">
         <v>100</v>
       </c>
-      <c r="C104" s="30"/>
-      <c r="D104" s="30"/>
-      <c r="E104" s="31"/>
+      <c r="C104" s="28"/>
+      <c r="D104" s="28"/>
+      <c r="E104" s="29"/>
       <c r="F104" s="3">
         <v>6</v>
       </c>
@@ -3823,128 +3873,123 @@
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="M104" s="51"/>
+      <c r="M104" s="45"/>
     </row>
     <row r="105" spans="1:13" ht="21.6" thickBot="1">
-      <c r="A105" s="36">
+      <c r="A105" s="34">
         <v>25</v>
       </c>
-      <c r="B105" s="17" t="s">
+      <c r="B105" s="35" t="s">
         <v>101</v>
       </c>
-      <c r="C105" s="22"/>
-      <c r="D105" s="22"/>
-      <c r="E105" s="23"/>
-      <c r="F105" s="4">
+      <c r="C105" s="36"/>
+      <c r="D105" s="36"/>
+      <c r="E105" s="37"/>
+      <c r="F105" s="46">
         <v>12</v>
       </c>
-      <c r="G105" s="4">
-        <v>6</v>
-      </c>
-      <c r="H105" s="3">
+      <c r="G105" s="46">
+        <v>6</v>
+      </c>
+      <c r="H105" s="46">
         <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="I105" s="4"/>
-      <c r="J105" s="4"/>
-      <c r="K105" s="4"/>
-      <c r="L105" s="3">
+      <c r="I105" s="46"/>
+      <c r="J105" s="46"/>
+      <c r="K105" s="46"/>
+      <c r="L105" s="46">
         <f t="shared" si="3"/>
         <v>6</v>
       </c>
-      <c r="M105" s="54"/>
+      <c r="M105" s="47"/>
     </row>
     <row r="106" spans="1:13" ht="21.6" thickBot="1">
-      <c r="A106" s="42" t="s">
+      <c r="A106" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B106" s="41" t="s">
+      <c r="B106" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="C106" s="41"/>
-      <c r="D106" s="41"/>
-      <c r="E106" s="41"/>
-      <c r="F106" s="44" t="s">
+      <c r="C106" s="48"/>
+      <c r="D106" s="48"/>
+      <c r="E106" s="48"/>
+      <c r="F106" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="G106" s="44" t="s">
+      <c r="G106" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="H106" s="44" t="s">
+      <c r="H106" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="I106" s="44" t="s">
-        <v>6</v>
-      </c>
-      <c r="J106" s="44" t="s">
+      <c r="I106" s="39" t="s">
+        <v>6</v>
+      </c>
+      <c r="J106" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="K106" s="44" t="s">
+      <c r="K106" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="L106" s="44" t="s">
+      <c r="L106" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="M106" s="48" t="s">
+      <c r="M106" s="42" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="107" spans="1:13">
-      <c r="A107" s="36">
+      <c r="A107" s="33">
         <v>26</v>
       </c>
-      <c r="B107" s="55" t="s">
+      <c r="B107" s="57" t="s">
         <v>67</v>
       </c>
-      <c r="C107" s="56"/>
-      <c r="D107" s="56"/>
-      <c r="E107" s="57"/>
-      <c r="F107" s="49">
-        <v>6</v>
-      </c>
-      <c r="G107" s="49">
+      <c r="C107" s="58"/>
+      <c r="D107" s="58"/>
+      <c r="E107" s="59"/>
+      <c r="F107" s="43">
+        <v>6</v>
+      </c>
+      <c r="G107" s="43">
         <v>3</v>
       </c>
-      <c r="H107" s="49">
+      <c r="H107" s="43">
         <v>3</v>
       </c>
-      <c r="I107" s="49"/>
-      <c r="J107" s="49"/>
-      <c r="K107" s="49"/>
-      <c r="L107" s="49">
+      <c r="I107" s="43"/>
+      <c r="J107" s="43"/>
+      <c r="K107" s="43"/>
+      <c r="L107" s="43">
         <v>3</v>
       </c>
-      <c r="M107" s="50"/>
+      <c r="M107" s="44"/>
     </row>
     <row r="108" spans="1:13">
-      <c r="A108" s="36">
+      <c r="A108" s="33">
         <v>27</v>
       </c>
-      <c r="B108" s="26" t="s">
+      <c r="B108" s="24" t="s">
         <v>102</v>
       </c>
-      <c r="C108" s="5"/>
-      <c r="D108" s="5"/>
-      <c r="E108" s="5"/>
-      <c r="F108" s="49"/>
-      <c r="G108" s="49"/>
-      <c r="H108" s="49"/>
-      <c r="I108" s="49"/>
-      <c r="J108" s="49"/>
-      <c r="K108" s="49"/>
-      <c r="L108" s="49"/>
-      <c r="M108" s="50"/>
+      <c r="F108" s="43"/>
+      <c r="G108" s="43"/>
+      <c r="H108" s="43"/>
+      <c r="I108" s="43"/>
+      <c r="J108" s="43"/>
+      <c r="K108" s="43"/>
+      <c r="L108" s="43"/>
+      <c r="M108" s="44"/>
     </row>
     <row r="109" spans="1:13">
-      <c r="A109" s="36"/>
-      <c r="B109" s="12" t="s">
+      <c r="A109" s="33"/>
+      <c r="B109" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C109" s="5" t="s">
+      <c r="C109" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="D109" s="5"/>
-      <c r="E109" s="5"/>
       <c r="F109" s="3">
         <v>6</v>
       </c>
@@ -3962,18 +4007,16 @@
         <f t="shared" ref="L109:L115" si="11">G109</f>
         <v>6</v>
       </c>
-      <c r="M109" s="51"/>
+      <c r="M109" s="45"/>
     </row>
     <row r="110" spans="1:13">
-      <c r="A110" s="36"/>
-      <c r="B110" s="12" t="s">
+      <c r="A110" s="33"/>
+      <c r="B110" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C110" s="5" t="s">
+      <c r="C110" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="D110" s="5"/>
-      <c r="E110" s="5"/>
       <c r="F110" s="3">
         <v>6</v>
       </c>
@@ -3991,18 +4034,18 @@
         <f t="shared" si="11"/>
         <v>5</v>
       </c>
-      <c r="M110" s="51"/>
+      <c r="M110" s="45"/>
     </row>
     <row r="111" spans="1:13">
-      <c r="A111" s="36"/>
-      <c r="B111" s="14" t="s">
+      <c r="A111" s="33"/>
+      <c r="B111" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C111" s="24" t="s">
+      <c r="C111" s="22" t="s">
         <v>104</v>
       </c>
-      <c r="D111" s="24"/>
-      <c r="E111" s="24"/>
+      <c r="D111" s="22"/>
+      <c r="E111" s="22"/>
       <c r="F111" s="3">
         <v>6</v>
       </c>
@@ -4020,18 +4063,18 @@
         <f t="shared" si="11"/>
         <v>4</v>
       </c>
-      <c r="M111" s="51"/>
+      <c r="M111" s="45"/>
     </row>
     <row r="112" spans="1:13">
-      <c r="A112" s="36">
+      <c r="A112" s="33">
         <v>28</v>
       </c>
-      <c r="B112" s="29" t="s">
+      <c r="B112" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="C112" s="30"/>
-      <c r="D112" s="30"/>
-      <c r="E112" s="31"/>
+      <c r="C112" s="28"/>
+      <c r="D112" s="28"/>
+      <c r="E112" s="29"/>
       <c r="F112" s="3">
         <v>6</v>
       </c>
@@ -4049,43 +4092,35 @@
         <f t="shared" si="11"/>
         <v>3</v>
       </c>
-      <c r="M112" s="51"/>
+      <c r="M112" s="45"/>
     </row>
     <row r="113" spans="1:13">
-      <c r="A113" s="36">
+      <c r="A113" s="33">
         <v>29</v>
       </c>
-      <c r="B113" s="17" t="s">
+      <c r="B113" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="C113" s="22"/>
-      <c r="D113" s="22"/>
-      <c r="E113" s="22"/>
+      <c r="C113" s="20"/>
+      <c r="D113" s="20"/>
+      <c r="E113" s="20"/>
       <c r="F113" s="3"/>
       <c r="G113" s="3"/>
-      <c r="H113" s="3">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
+      <c r="H113" s="3"/>
       <c r="I113" s="3"/>
       <c r="J113" s="3"/>
       <c r="K113" s="3"/>
-      <c r="L113" s="3">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="M113" s="51"/>
+      <c r="L113" s="3"/>
+      <c r="M113" s="45"/>
     </row>
     <row r="114" spans="1:13">
-      <c r="A114" s="36"/>
-      <c r="B114" s="12" t="s">
+      <c r="A114" s="33"/>
+      <c r="B114" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C114" s="5" t="s">
+      <c r="C114" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="D114" s="5"/>
-      <c r="E114" s="5"/>
       <c r="F114" s="3">
         <v>2</v>
       </c>
@@ -4103,36 +4138,36 @@
         <f t="shared" si="11"/>
         <v>2</v>
       </c>
-      <c r="M114" s="51"/>
+      <c r="M114" s="45"/>
     </row>
     <row r="115" spans="1:13" ht="21.6" thickBot="1">
-      <c r="A115" s="37"/>
-      <c r="B115" s="46" t="s">
+      <c r="A115" s="34"/>
+      <c r="B115" s="40" t="s">
         <v>61</v>
       </c>
-      <c r="C115" s="47" t="s">
+      <c r="C115" s="41" t="s">
         <v>108</v>
       </c>
-      <c r="D115" s="47"/>
-      <c r="E115" s="47"/>
-      <c r="F115" s="52">
+      <c r="D115" s="41"/>
+      <c r="E115" s="41"/>
+      <c r="F115" s="46">
         <v>1</v>
       </c>
-      <c r="G115" s="52">
+      <c r="G115" s="46">
         <v>1</v>
       </c>
-      <c r="H115" s="52">
+      <c r="H115" s="46">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="I115" s="52"/>
-      <c r="J115" s="52"/>
-      <c r="K115" s="52"/>
-      <c r="L115" s="52">
+      <c r="I115" s="46"/>
+      <c r="J115" s="46"/>
+      <c r="K115" s="46"/>
+      <c r="L115" s="46">
         <f t="shared" si="11"/>
         <v>1</v>
       </c>
-      <c r="M115" s="53"/>
+      <c r="M115" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>